<commit_message>
docs: colonne « Concept OpenMRS » dans le dictionnaire de données
Ajoute à chaque feuille-table une colonne « Concept OpenMRS (libellé + UUID) »
mappant les colonnes du hub au concept OpenMRS source, extrait des constantes
_UUID des extracteurs sync (commentaires = libellés FR). Rempli pour les
mappings directs (poids, CV, CD4, régime ARV, stades, TPT, dates ARV…) ;
colonnes techniques ou dérivées laissées vides. Ex. visits : 21 concepts.

Pertinent pour les analystes qui connaissent la source OpenMRS. Mapping maintenu
dans gen_dico.py (dict CONCEPTS).
</commit_message>
<xml_diff>
--- a/docs/SIGDEP3_dictionnaire_donnees.xlsx
+++ b/docs/SIGDEP3_dictionnaire_donnees.xlsx
@@ -865,15 +865,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -921,6 +922,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -953,6 +959,7 @@
           <t>Initiation parente (FK → treatment_initiations.id, lien 1-1). Clé primaire.</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -977,6 +984,7 @@
           <t>Poids de naissance (kg).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1001,6 +1009,7 @@
           <t>Taille de naissance (cm).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1025,6 +1034,7 @@
           <t>Périmètre crânien (cm).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1049,6 +1059,7 @@
           <t>Score d'Apgar.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1073,6 +1084,7 @@
           <t>Mode d'accouchement.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1097,6 +1109,7 @@
           <t>Accouchement en structure de santé.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1121,6 +1134,7 @@
           <t>La mère a reçu la PTME.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1145,6 +1159,7 @@
           <t>Statut VIH de la mère.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1169,6 +1184,7 @@
           <t>Statut vital de la mère.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1193,6 +1209,7 @@
           <t>Régime PTME de la mère.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1217,6 +1234,7 @@
           <t>Prophylaxie ARV donnée au nourrisson.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1241,6 +1259,7 @@
           <t>Protocole ARV du nourrisson.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1265,6 +1284,7 @@
           <t>Mode d'alimentation du nourrisson.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1289,6 +1309,7 @@
           <t>Date de sevrage.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1313,6 +1334,7 @@
           <t>Vaccinations reçues.</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1337,6 +1359,7 @@
           <t>Statut vital du père</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1361,6 +1384,7 @@
           <t>Niveau d'éducation du père</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1385,6 +1409,7 @@
           <t>Type d'activité du père</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1409,6 +1434,7 @@
           <t>Niveau d'éducation du mère</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1433,6 +1459,7 @@
           <t>Type d'activité du mère</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1457,6 +1484,7 @@
           <t>Statut vital du tuteur</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1481,6 +1509,7 @@
           <t>Niveau d'éducation du tuteur</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1505,6 +1534,7 @@
           <t>Type d'activité du tuteur</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1529,6 +1559,7 @@
           <t>Statut VIH du tuteur</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1553,6 +1584,7 @@
           <t>Date d'admission.</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1577,6 +1609,7 @@
           <t>Statut de scolarisation.</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1601,6 +1634,7 @@
           <t>Code de dépistage associé.</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1629,6 +1663,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1657,10 +1692,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1672,15 +1708,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1728,6 +1765,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -1760,6 +1802,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1792,6 +1835,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1824,6 +1868,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1852,6 +1897,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1876,6 +1922,7 @@
           <t>Formulaire OpenMRS d'origine de la visite (ex. « PEC - Suivi patient »).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1904,6 +1951,7 @@
           <t>Date de la visite. Clé de PARTITIONNEMENT de la table. Borne des vues « période ».</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1928,6 +1976,12 @@
           <t>Date du prochain rendez-vous.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Date de la prochaine visite
+5096AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1952,6 +2006,7 @@
           <t>Résultat du dépistage TB à la visite.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1976,6 +2031,7 @@
           <t>Tuberculose diagnostiquée (booléen).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2000,6 +2056,7 @@
           <t>Statut du traitement TB.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2024,6 +2081,7 @@
           <t>Date de début du traitement TB.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2048,6 +2106,12 @@
           <t>Stade clinique OMS (1 à 4) à la visite.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Stade clinique OMS (courant)
+5356AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2072,6 +2136,7 @@
           <t>Stade CDC à la visite.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2096,6 +2161,7 @@
           <t>Cotrimoxazole prescrit (booléen).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2120,6 +2186,7 @@
           <t>Date de début du cotrimoxazole.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2144,6 +2211,7 @@
           <t>IVSA — date de confirmation de succès (suivi des non-stables).</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2168,6 +2236,7 @@
           <t>Patiente enceinte à la visite.</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2192,6 +2261,12 @@
           <t>Patiente allaitante à la visite.</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Allaitement en cours
+164764AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2216,6 +2291,12 @@
           <t>Poids (kg).</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Poids (kg)
+5089AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2240,6 +2321,12 @@
           <t>Taille (cm).</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Taille (cm)
+5090AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2264,6 +2351,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2288,6 +2376,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2316,6 +2405,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2344,6 +2434,7 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2368,6 +2459,12 @@
           <t>Régime ARV en cours (ex. TDF 3TC DTG). Sert aussi à la vue Pharmacie.</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Régime ARV
+162240AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2392,6 +2489,12 @@
           <t>Température (°C).</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Température (°C)
+5088AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2416,6 +2519,12 @@
           <t>Pouls (battements/min).</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Pouls
+5087AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2440,6 +2549,12 @@
           <t>Fréquence respiratoire (cycles/min).</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Rythme respiratoire
+5242AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2464,6 +2579,12 @@
           <t>Tension artérielle systolique (mmHg).</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Tension artérielle systolique
+5085AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2488,6 +2609,12 @@
           <t>Tension artérielle diastolique (mmHg).</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Tension artérielle diastolique
+5086AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2512,6 +2639,12 @@
           <t>Indice de masse corporelle (calculé).</t>
         </is>
       </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>IMC
+1342AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -2536,6 +2669,12 @@
           <t>Périmètre brachial (cm).</t>
         </is>
       </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Périmètre brachial
+163586AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -2560,6 +2699,12 @@
           <t>Charge virale (copies/mL) relevée à la visite.</t>
         </is>
       </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>VIH charge virale
+856AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2584,6 +2729,12 @@
           <t>Date de la charge virale.</t>
         </is>
       </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Date dernière charge virale
+165015AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2608,6 +2759,12 @@
           <t>Taux de CD4 (cellules/µL) relevé à la visite.</t>
         </is>
       </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>CD4 (patient reported)
+159375AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2632,6 +2789,12 @@
           <t>Date du CD4.</t>
         </is>
       </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Date du dernier CD4
+160103AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2656,6 +2819,12 @@
           <t>Nombre de jours d'ARV dispensés (durée de couverture).</t>
         </is>
       </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Nombre de jours de traitement ARV
+164590AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2680,6 +2849,12 @@
           <t>Nombre de jours de cotrimoxazole dispensés.</t>
         </is>
       </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Nombre de jours de cotrimoxazole
+164578AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2704,6 +2879,7 @@
           <t>Statut d'allaitement.</t>
         </is>
       </c>
+      <c r="G43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2728,6 +2904,12 @@
           <t>Statut TPT à la visite.</t>
         </is>
       </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Traitement TPT (statut)
+165049AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2752,6 +2934,12 @@
           <t>Protocole TPT à la visite.</t>
         </is>
       </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Protocole TPT
+165319AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2776,6 +2964,7 @@
           <t>IVSA — code MSD (motif/signe).</t>
         </is>
       </c>
+      <c r="G46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2800,6 +2989,7 @@
           <t>IVSA — nombre de signes d'alerte.</t>
         </is>
       </c>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -2824,10 +3014,11 @@
           <t>IVSA — nombre de signes neurologiques.</t>
         </is>
       </c>
+      <c r="G48" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2839,15 +3030,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2895,6 +3087,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -2927,6 +3124,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2959,6 +3157,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2991,6 +3190,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -3019,6 +3219,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3043,6 +3244,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3063,6 +3265,7 @@
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3083,6 +3286,7 @@
       <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3103,6 +3307,7 @@
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -3123,6 +3328,7 @@
       <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="5" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3147,6 +3353,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3171,6 +3378,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3199,6 +3407,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3227,10 +3436,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3242,15 +3452,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3298,6 +3509,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -3330,6 +3546,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3362,6 +3579,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3394,6 +3612,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -3426,6 +3645,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3454,6 +3674,7 @@
           <t>UUID de l'encounter (bilan) d'origine — regroupe les résultats d'un même bilan.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3482,6 +3703,7 @@
           <t>UUID du concept OpenMRS de l'examen (identifie le type d'examen).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3506,6 +3728,7 @@
           <t>Libellé de l'examen (ex. VIH CHARGE VIRALE, CRÉATININE, CD4).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3530,6 +3753,7 @@
           <t>Date de l'examen. Indexée pour les vues nationales (idx_lab_exam_date).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -3554,6 +3778,7 @@
           <t>Résultat numérique (le plus fréquent).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3578,6 +3803,7 @@
           <t>Résultat texte libre (ex. « &lt; LL »).</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3602,6 +3828,7 @@
           <t>Résultat codé : libellé de la réponse (Positif/Négatif/Détectable…). Utilisé pour les examens qualitatifs (Type VIH, HBs, CV qualitative).</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3626,6 +3853,7 @@
           <t>Unité de mesure du résultat numérique.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3650,6 +3878,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3678,6 +3907,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -3706,10 +3936,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3721,15 +3952,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3777,6 +4009,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -3809,6 +4046,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3841,6 +4079,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3873,6 +4112,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -3905,6 +4145,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3929,6 +4170,7 @@
           <t>Type de clôture : DEATH (décès), TRANSFER (transfert), et arrêt volontaire / sérologie négative selon les dates renseignées.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3953,6 +4195,7 @@
           <t>Date de clôture du dossier.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3977,6 +4220,12 @@
           <t>Date de transfert (si transfert).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Date de transfert
+164595AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -4001,6 +4250,12 @@
           <t>Structure de destination du transfert.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Destination du transfert
+164665AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -4025,6 +4280,12 @@
           <t>Motif du transfert.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Motif du transfert
+165216AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -4049,6 +4310,12 @@
           <t>Date de décès déclarée.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Date de décès
+1543AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -4073,6 +4340,12 @@
           <t>Date de décès réelle/constatée.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Date de décès réelle
+165233AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -4097,6 +4370,12 @@
           <t>Cause de décès (codée).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Cause de décès (codée)
+165225AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -4121,6 +4400,12 @@
           <t>Cause de décès (texte libre).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Cause de décès (texte)
+162580AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -4145,6 +4430,7 @@
           <t>Date d'arrêt volontaire du traitement.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -4169,6 +4455,7 @@
           <t>Date d'infirmation du statut VIH (clôture pour sérologie négative).</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -4193,6 +4480,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -4217,6 +4505,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -4245,6 +4534,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -4273,10 +4563,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4288,15 +4579,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4344,6 +4636,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -4376,6 +4673,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -4408,6 +4706,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -4440,6 +4739,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -4468,6 +4768,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -4496,6 +4797,7 @@
           <t>Nature de l'enregistrement TPT (démarrage / suivi / fin).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -4520,6 +4822,7 @@
           <t>Date de l'enregistrement (borne des vues « période »).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -4544,6 +4847,12 @@
           <t>Date de suivi TPT.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Date de visite TPT
+165234AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -4568,6 +4877,12 @@
           <t>Date de fin du TPT.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Date de fin du TPT
+165202AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -4592,6 +4907,7 @@
           <t>Issue du TPT (terminé, interrompu…).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -4616,6 +4932,12 @@
           <t>Numéro d'ordre/prescription TPT.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Numéro d'ordre TPT
+165244AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -4640,6 +4962,12 @@
           <t>Observance au TPT.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Observance traitement préventif
+165200AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -4664,6 +4992,12 @@
           <t>Poids (kg) au moment de l'enregistrement.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Poids (kg)
+5089AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -4688,6 +5022,7 @@
           <t>Date de la prochaine visite.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -4712,6 +5047,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -4736,6 +5072,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -4764,6 +5101,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -4792,6 +5130,7 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -4816,6 +5155,12 @@
           <t>Statut du TPT.</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Traitement TPT (statut)
+165049AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -4840,10 +5185,16 @@
           <t>Protocole TPT (ex. INH, 3HP).</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Protocole TPT
+165319AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4855,15 +5206,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4911,6 +5263,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -4943,6 +5300,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -4975,6 +5333,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -5003,6 +5362,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -5027,6 +5387,7 @@
           <t>Code du dépistage.</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -5051,6 +5412,7 @@
           <t>Date du dépistage (borne des vues « période »).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -5075,6 +5437,7 @@
           <t>Date d'annonce du résultat.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -5099,6 +5462,7 @@
           <t>Sexe de la personne dépistée.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -5123,6 +5487,7 @@
           <t>Âge au dépistage.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -5147,6 +5512,7 @@
           <t>Profession.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -5171,6 +5537,7 @@
           <t>Résidence.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -5195,6 +5562,7 @@
           <t>Situation matrimoniale.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -5219,6 +5587,7 @@
           <t>Précision si « autre » situation matrimoniale.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -5243,6 +5612,7 @@
           <t>Type de population (générale, clé…).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -5267,6 +5637,7 @@
           <t>Motif du dépistage.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -5291,6 +5662,7 @@
           <t>Précision si « autre » motif.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -5315,6 +5687,7 @@
           <t>Réaction du test 1 (R/NR).</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -5339,6 +5712,7 @@
           <t>Réaction du test 2.</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -5363,6 +5737,7 @@
           <t>Réaction du test 3.</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -5387,6 +5762,7 @@
           <t>Test 1 invalidé.</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -5411,6 +5787,7 @@
           <t>Test 2 invalidé.</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -5435,6 +5812,7 @@
           <t>Test 3 invalidé.</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -5459,6 +5837,7 @@
           <t>Résultat final du dépistage (POS/NEG/IND).</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -5483,6 +5862,7 @@
           <t>Re-test effectué.</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -5507,6 +5887,7 @@
           <t>Commentaire libre.</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -5531,6 +5912,7 @@
           <t>Type de site de dépistage (porte d'entrée).</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -5555,6 +5937,7 @@
           <t>Poste de dépistage.</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -5579,6 +5962,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -5603,6 +5987,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -5631,6 +6016,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -5659,10 +6045,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5674,15 +6061,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5730,6 +6118,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -5762,6 +6155,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -5794,6 +6188,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -5822,6 +6217,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -5846,6 +6242,7 @@
           <t>Numéro de suivi grossesse.</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -5870,6 +6267,7 @@
           <t>Numéro de prise en charge VIH.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -5894,6 +6292,7 @@
           <t>Numéro de dépistage.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -5918,6 +6317,7 @@
           <t>Âge de la mère.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -5942,6 +6342,7 @@
           <t>Situation matrimoniale.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -5966,6 +6367,7 @@
           <t>Dépistage du conjoint (réalisé/non).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -5990,6 +6392,7 @@
           <t>Résultat du dépistage conjoint.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -6014,6 +6417,7 @@
           <t>Date de début de suivi PTME. Souvent NULL (81 %) → fiches invisibles en vue « période ».</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -6038,6 +6442,7 @@
           <t>Date de fin de suivi.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -6062,6 +6467,7 @@
           <t>Statut ARV à l'inscription.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -6086,6 +6492,7 @@
           <t>Date prévue d'accouchement.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -6110,6 +6517,7 @@
           <t>Issue de la grossesse.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -6134,6 +6542,7 @@
           <t>Date du dépistage conjoint.</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -6158,6 +6567,7 @@
           <t>Type d'accouchement.</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -6182,6 +6592,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -6206,6 +6617,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -6234,6 +6646,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -6262,10 +6675,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6277,15 +6691,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6333,6 +6748,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -6365,6 +6785,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -6397,6 +6818,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -6425,6 +6847,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -6449,6 +6872,7 @@
           <t>UUID source de la mère (rattachement).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -6473,6 +6897,7 @@
           <t>Date de la visite.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -6497,6 +6922,7 @@
           <t>Âge gestationnel (semaines).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -6521,6 +6947,7 @@
           <t>Poursuite des ARV (O/N/NA).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -6545,6 +6972,7 @@
           <t>Poursuite du cotrimoxazole (O/N/NA).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -6569,6 +6997,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -6593,6 +7022,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -6621,6 +7051,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -6649,10 +7080,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6664,15 +7096,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6720,6 +7153,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -6752,6 +7190,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -6784,6 +7223,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -6812,6 +7252,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -6836,6 +7277,7 @@
           <t>UUID source de la mère (lien enfant → mère).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -6860,6 +7302,7 @@
           <t>Numéro de suivi de l'enfant.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -6884,6 +7327,7 @@
           <t>Date de naissance de l'enfant.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -6908,6 +7352,7 @@
           <t>Sexe de l'enfant.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -6932,6 +7377,7 @@
           <t>Prophylaxie ARV donnée (O/N/NA).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -6956,6 +7402,7 @@
           <t>Date de la prophylaxie ARV.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -6980,6 +7427,7 @@
           <t>Date de fin de suivi.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -7004,6 +7452,7 @@
           <t>Date de prélèvement (PCR1).</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -7028,6 +7477,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -7052,6 +7502,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -7076,6 +7527,7 @@
           <t>Résultat PCR 1 (POS/NEG…).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -7100,6 +7552,7 @@
           <t>Date de prélèvement (PCR2).</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -7124,6 +7577,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -7148,6 +7602,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -7172,6 +7627,7 @@
           <t>Résultat PCR 2.</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -7196,6 +7652,7 @@
           <t>Date de prélèvement (PCR3).</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -7220,6 +7677,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -7244,6 +7702,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -7268,6 +7727,7 @@
           <t>Résultat PCR 3.</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -7292,6 +7752,7 @@
           <t>Date d'initiation (CTX).</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -7316,6 +7777,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -7340,6 +7802,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -7364,6 +7827,7 @@
           <t>Date d'initiation (INH).</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -7388,6 +7852,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -7412,6 +7877,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -7436,6 +7902,7 @@
           <t>Date de la sérologie VIH.</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -7460,6 +7927,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -7484,6 +7952,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -7508,6 +7977,7 @@
           <t>Résultat sérologie VIH 1.</t>
         </is>
       </c>
+      <c r="G36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -7532,6 +8002,7 @@
           <t>Date de la sérologie VIH.</t>
         </is>
       </c>
+      <c r="G37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -7556,6 +8027,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -7580,6 +8052,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -7604,6 +8077,7 @@
           <t>Résultat sérologie VIH 2.</t>
         </is>
       </c>
+      <c r="G40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -7628,6 +8102,7 @@
           <t>Résultat final du suivi de l'enfant.</t>
         </is>
       </c>
+      <c r="G41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -7652,6 +8127,7 @@
           <t>Date du résultat final.</t>
         </is>
       </c>
+      <c r="G42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -7676,6 +8152,7 @@
           <t>Lieu de référence.</t>
         </is>
       </c>
+      <c r="G43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -7700,6 +8177,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -7724,6 +8202,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -7752,6 +8231,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -7780,10 +8260,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7931,15 +8412,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7987,6 +8469,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -8019,6 +8506,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -8051,6 +8539,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -8079,6 +8568,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -8103,6 +8593,7 @@
           <t>UUID source de l'enfant (rattachement).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -8127,6 +8618,7 @@
           <t>Date de la visite.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -8151,6 +8643,7 @@
           <t>Âge de l'enfant en jours à l'événement.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -8175,6 +8668,7 @@
           <t>Âge de l'enfant en semaines à l'événement.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -8199,6 +8693,7 @@
           <t>Âge de l'enfant en mois à l'événement.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -8223,6 +8718,7 @@
           <t>Mode d'alimentation.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -8247,6 +8743,7 @@
           <t>Méthode contraceptive moderne (contexte).</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -8271,6 +8768,7 @@
           <t>Poursuite du cotrimoxazole.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -8295,6 +8793,7 @@
           <t>Poursuite de l'INH (prophylaxie TB).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -8319,6 +8818,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -8343,6 +8843,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -8371,6 +8872,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -8399,10 +8901,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8414,15 +8917,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8470,6 +8974,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -8502,6 +9011,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -8530,6 +9040,7 @@
           <t>Code de la région (référentiel national).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -8558,6 +9069,7 @@
           <t>Libellé de la région.</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -8582,6 +9094,7 @@
           <t>UUID de référence (facultatif).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -8610,6 +9123,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -8638,10 +9152,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8653,15 +9168,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8709,6 +9225,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -8741,6 +9262,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -8769,6 +9291,7 @@
           <t>Code du district.</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -8801,6 +9324,7 @@
           <t>Région de rattachement (FK → regions.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -8829,6 +9353,7 @@
           <t>Libellé du district.</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -8853,6 +9378,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -8881,6 +9407,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -8909,10 +9436,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8924,15 +9452,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8980,6 +9509,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -9012,6 +9546,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -9040,6 +9575,7 @@
           <t>Code établissement (ex. 00064). Correspond à SIGDEP_SITE_CODE côté agent.</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -9068,6 +9604,7 @@
           <t>Nom de l'établissement.</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -9100,6 +9637,7 @@
           <t>District de rattachement (FK → districts.id).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -9124,6 +9662,7 @@
           <t>Type d'établissement (CSU, HG, CHR…).</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -9148,6 +9687,7 @@
           <t>Latitude géographique (décimale).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -9172,6 +9712,7 @@
           <t>Longitude géographique (décimale).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -9196,6 +9737,7 @@
           <t>Site actif dans la plateforme.</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -9220,6 +9762,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -9244,6 +9787,7 @@
           <t>Empreinte (hash) de la clé API du site pour l'ingestion. Technique/sécurité.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -9268,6 +9812,7 @@
           <t>Date-heure de la dernière synchronisation reçue de ce site.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -9296,6 +9841,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -9324,6 +9870,7 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -9348,10 +9895,11 @@
           <t>Le site fait-il effectivement tourner un agent SIGDEP (vs site référencé sans agent).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9363,15 +9911,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9419,6 +9968,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -9451,6 +10005,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -9479,6 +10034,7 @@
           <t>Code du type d'identifiant (UPID, CODE_ARV, CRUID, UPID…).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -9507,6 +10063,7 @@
           <t>Libellé du type d'identifiant.</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -9531,6 +10088,7 @@
           <t>Description du type.</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -9555,6 +10113,7 @@
           <t>Expression régulière de validation du format attendu.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -9579,10 +10138,11 @@
           <t>Type d'identifiant actif.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9594,15 +10154,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9650,6 +10211,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -9682,6 +10248,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -9714,6 +10281,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -9746,6 +10314,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -9770,6 +10339,7 @@
           <t>Sexe : 'M' (masculin), 'F' (féminin), 'U' (inconnu).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -9794,6 +10364,7 @@
           <t>Date de naissance.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -9818,6 +10389,7 @@
           <t>Vrai si la date de naissance est estimée (jour/mois par défaut).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -9842,6 +10414,12 @@
           <t>Lieu de naissance (texte libre issu de la source).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Lieu de naissance
+164444AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -9866,6 +10444,12 @@
           <t>Profession (texte).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Profession
+162904AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -9890,6 +10474,12 @@
           <t>Niveau d'éducation.</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Niveau d'éducation
+1712AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -9914,6 +10504,12 @@
           <t>Situation matrimoniale.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>État civil
+1054AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -9938,6 +10534,12 @@
           <t>Religion.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Religion
+162894AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -9962,6 +10564,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -9986,6 +10589,7 @@
           <t>Date-heure de la suppression logique du patient (si voided).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -10014,6 +10618,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -10042,10 +10647,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10057,15 +10663,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10113,6 +10720,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -10145,6 +10757,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -10177,6 +10790,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -10209,6 +10823,7 @@
           <t>Type d'identifiant (FK → identifier_types.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -10237,6 +10852,7 @@
           <t>Valeur de l'identifiant (ex. code ARV, UPID).</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -10261,6 +10877,7 @@
           <t>Identifiant préféré/principal pour ce patient.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -10293,6 +10910,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -10317,6 +10935,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -10341,6 +10960,7 @@
           <t>Début de validité (facultatif).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -10365,6 +10985,7 @@
           <t>Fin de validité (facultatif).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -10389,6 +11010,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -10417,6 +11039,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -10445,10 +11068,11 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10460,15 +11084,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10516,6 +11141,11 @@
           <t>Description métier</t>
         </is>
       </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Concept OpenMRS (libellé + UUID)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -10548,6 +11178,7 @@
           <t>Identifiant technique interne (clé primaire, auto-incrément). Sans signification métier.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -10580,6 +11211,7 @@
           <t>Patient concerné (FK → patients.id).</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -10612,6 +11244,7 @@
           <t>Site d'appartenance de l'enregistrement (FK → sites.id).</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -10644,6 +11277,7 @@
           <t>UUID d'origine dans la base OpenMRS du site. Unique PAR SITE (couple site_id, source_uuid).</t>
         </is>
       </c>
+      <c r="G8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -10668,6 +11302,7 @@
           <t>Date d'enrôlement dans la file active. Sert de repli quand arv_init_date est absente.</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -10692,6 +11327,12 @@
           <t>Date de mise sous ARV. NULL fréquent (~64 %) → les vues « période » retombent sur enrollment_date.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Date de début ARV
+159599AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -10716,6 +11357,12 @@
           <t>Date du test VIH.</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Date diagnostique VIH
+160554AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -10740,6 +11387,12 @@
           <t>Type de VIH (VIH-1, VIH-2, VIH-1&amp;2).</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Résultat Type VIH
+163623AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -10764,6 +11417,12 @@
           <t>Porte d'entrée dans les soins (consultation, PTME, dépistage…).</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Point d'entrée
+164523AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -10788,6 +11447,7 @@
           <t>Données additionnelles non modélisées, au format JSON (paires concept OpenMRS → valeur). Champ d'extension.</t>
         </is>
       </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -10812,6 +11472,7 @@
           <t>Vrai = enregistrement supprimé logiquement (exclu de toutes les statistiques). Défaut : faux.</t>
         </is>
       </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -10840,6 +11501,7 @@
           <t>Horodatage d'insertion dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -10868,6 +11530,7 @@
           <t>Horodatage de dernière mise à jour dans le hub (technique).</t>
         </is>
       </c>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -10892,6 +11555,12 @@
           <t>Stade clinique OMS à l'initiation (I à IV).</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Stade clinique OMS
+164487AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -10916,6 +11585,12 @@
           <t>Stade CDC à l'initiation.</t>
         </is>
       </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Stadification CDC
+1209AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -10940,6 +11615,12 @@
           <t>Régime ARV initial (ex. TDF 3TC DTG).</t>
         </is>
       </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Régime ARV
+162240AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -10964,6 +11645,12 @@
           <t>Poids à l'initiation (kg).</t>
         </is>
       </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Poids (kg)
+5089AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -10988,6 +11675,12 @@
           <t>Taux de CD4 à l'initiation (cellules/µL).</t>
         </is>
       </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Numération CD4
+5497AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -11012,6 +11705,12 @@
           <t>Pourcentage de CD4 à l'initiation.</t>
         </is>
       </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>CD4%
+730AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -11036,6 +11735,12 @@
           <t>Indice de Karnofsky (état général, 0–100).</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Score de Karnofsky
+5283AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -11060,6 +11765,12 @@
           <t>Patient référé (Oui/Non).</t>
         </is>
       </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Patient référé
+1648AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -11084,6 +11795,12 @@
           <t>Origine de la référence.</t>
         </is>
       </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Référé origine
+164562AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -11108,6 +11825,12 @@
           <t>Motif du traitement.</t>
         </is>
       </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Motif mise sous TARV
+162225AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -11132,6 +11855,12 @@
           <t>Statut VIH du partenaire.</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Statut sérologique partenaire
+1436AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -11156,6 +11885,12 @@
           <t>Antécédent de tuberculose.</t>
         </is>
       </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Antécédent tuberculose
+1389AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -11180,6 +11915,12 @@
           <t>Antécédent de traitement ARV.</t>
         </is>
       </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Antécédent ARV
+164540AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -11204,6 +11945,12 @@
           <t>Antécédent de transfusion.</t>
         </is>
       </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Antécédent transfusion
+1871AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -11228,6 +11975,12 @@
           <t>Antécédent PTME.</t>
         </is>
       </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Antécédent PTME
+163450AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -11252,6 +12005,12 @@
           <t>Régime PTME antérieur.</t>
         </is>
       </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Régime antécédent PTME
+1400AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -11276,10 +12035,16 @@
           <t>Date de l'antécédent PTME.</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Date PTME
+164588AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>